<commit_message>
데미지 더하기 방식: CritMult→CritDamage, Skill DamageMult→Damage
10/29 개발·기획 회의 후 결정. 데미지는 정수 더하기만, 배율은 확률에만.
UnitStat CritDamage(막손 6, 허수귀 10, 지게귀 13, 변종 16, 보스 14),
Skill 7001 Damage 6. Item·Buff statType 목록과 README도 같이 고침.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CDH3mxXsBhjTgcPjfLvqYR
</commit_message>
<xml_diff>
--- a/tables/Buff.xlsx
+++ b/tables/Buff.xlsx
@@ -415,23 +415,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <ns0:sheetPr>
-    <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
-    <ns0:pageSetUpPr/>
-  </ns0:sheetPr>
-  <ns0:dimension ref="A1:K8"/>
-  <ns0:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <ns0:sheetData>
-    <ns0:row r="1">
-      <ns0:c r="A1" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>규칙</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B1" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">한 행 = 버프·회복 효과 하나(10/29 Player 탭에서 분리). Key enum: Heal(즉시 회복), StatAdd(일정 시간 스탯 더하기). StatType = UnitStat 열 이름(HP, ATK, DEF, Dodge, Crit, CritMult, Poise, MoveSpeed, ArmorPen). Value는 정수(비율 스탯은 만분율). Duration·TickInterval·UseTime은 ms, 0 = 즉시·한 번. Charges = 한 번 쉴 때 채워지는 사용 횟수(0 = 제한 없음). Stackable Y/N. 계산식은 Formula 탭.
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>규칙</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>한 행 = 버프·회복 효과 하나(10/29 Player 탭에서 분리). Key enum: Heal(즉시 회복), StatAdd(일정 시간 스탯 더하기). StatType = UnitStat 열 이름(HP, ATK, DEF, Dodge, Crit, CritDamage, Poise, MoveSpeed, ArmorPen). Value는 정수(비율 스탯은 만분율). Duration·TickInterval·UseTime은 ms, 0 = 즉시·한 번. Charges = 한 번 쉴 때 채워지는 사용 횟수(0 = 제한 없음). Stackable Y/N. 계산식은 Formula 탭.
 [추출 지정 규칙]
 @column Name=Key;Type=Text;AllowedValues=Heal|StatAdd
 @column Name=StatType;Type=Text;SharedStatKeysFrom=UnitStat
@@ -440,206 +440,206 @@
 @column Name=TickInterval;Type=Integer;Minimum=0;Unit=ms
 @column Name=UseTime;Type=Integer;Minimum=0;Unit=ms
 @column Name=Charges;Type=Integer;Minimum=0
-@column Name=Stackable;Type=Flag</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="2">
-      <ns0:c r="A2" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>기능</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B2" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>CSV,회복·버프 종류·수치·지속 시간·사용 횟수.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="3">
-      <ns0:c r="A3" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>역할</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B3" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>전투 코드의 버프·회복 처리, Item(Consumable)·Skill이 ID로 참조.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="4">
-      <ns0:c r="A4" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>의도</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B4" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>캐릭터 시트를 짧게 두고, 버프·회복 수치를 한 곳에서 행 추가로 관리하기 위해.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="5">
-      <ns0:c r="A5" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>비고</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B5" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Name, Note</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="6">
-      <ns0:c r="A6" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ID</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B6" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Name</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C6" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Key</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D6" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>StatType</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E6" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Value</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F6" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Duration</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="G6" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>TickInterval</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H6" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>UseTime</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="I6" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Charges</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="J6" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Stackable</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="K6" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Note</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="7">
-      <ns0:c r="A7" s="1" t="n">
-        <ns0:v>14001</ns0:v>
-      </ns0:c>
-      <ns0:c r="B7" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>약초 회복</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C7" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Heal</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D7" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>HP</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E7" s="1" t="n">
-        <ns0:v>40</ns0:v>
-      </ns0:c>
-      <ns0:c r="F7" s="1" t="n">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="G7" s="1" t="n">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="H7" s="1" t="n">
-        <ns0:v>800</ns0:v>
-      </ns0:c>
-      <ns0:c r="I7" s="1" t="n">
-        <ns0:v>3</ns0:v>
-      </ns0:c>
-      <ns0:c r="J7" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>N</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="K7" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>옛 Player.HerbHeal·HerbCount·HerbUseTime(10/29 이동). 지스타 약초</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="8">
-      <ns0:c r="A8" s="1" t="n">
-        <ns0:v>14002</ns0:v>
-      </ns0:c>
-      <ns0:c r="B8" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>공격 강화(예시)</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C8" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>StatAdd</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D8" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ATK</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E8" s="1" t="n">
-        <ns0:v>3</ns0:v>
-      </ns0:c>
-      <ns0:c r="F8" s="1" t="n">
-        <ns0:v>10000</ns0:v>
-      </ns0:c>
-      <ns0:c r="G8" s="1" t="n">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="H8" s="1" t="n">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="I8" s="1" t="n">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="J8" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>N</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="K8" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>구조 예시 행, 미확정</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-  </ns0:sheetData>
-  <ns0:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</ns0:worksheet>
+@column Name=Stackable;Type=Flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>기능</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>CSV,회복·버프 종류·수치·지속 시간·사용 횟수.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>역할</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>전투 코드의 버프·회복 처리, Item(Consumable)·Skill이 ID로 참조.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>의도</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>캐릭터 시트를 짧게 두고, 버프·회복 수치를 한 곳에서 행 추가로 관리하기 위해.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Name, Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>StatType</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>TickInterval</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>UseTime</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>Charges</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>Stackable</t>
+        </is>
+      </c>
+      <c r="K6" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>14001</v>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>약초 회복</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Heal</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>800</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K7" s="1" t="inlineStr">
+        <is>
+          <t>옛 Player.HerbHeal·HerbCount·HerbUseTime(10/29 이동). 지스타 약초</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>14002</v>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>공격 강화(예시)</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>StatAdd</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>ATK</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K8" s="1" t="inlineStr">
+        <is>
+          <t>구조 예시 행, 미확정</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>